<commit_message>
Update Excel report with distinct MRP and Selling Price
</commit_message>
<xml_diff>
--- a/full_product_variants_report.xlsx
+++ b/full_product_variants_report.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,45 +450,50 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Price (INR)</t>
+          <t>MRP (INR)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Selling Price (INR)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>How To Use</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Key Benefits</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Suitable For</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Specifications</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Badges</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Thumbnail</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Variant Image 1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Requires Attention</t>
         </is>
@@ -523,14 +528,17 @@
       <c r="F2" t="n">
         <v>299</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -539,32 +547,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -599,14 +607,17 @@
       <c r="F3" t="n">
         <v>299</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -615,32 +626,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Black.webp</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -675,14 +686,17 @@
       <c r="F4" t="n">
         <v>299</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -691,32 +705,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Light Brown.webp</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -751,14 +765,17 @@
       <c r="F5" t="n">
         <v>299</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -767,32 +784,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Medium Brown.webp</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -827,14 +844,17 @@
       <c r="F6" t="n">
         <v>299</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -843,32 +863,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Dark Brown.webp</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -903,14 +923,17 @@
       <c r="F7" t="n">
         <v>299</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -919,32 +942,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Tan.webp</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -979,14 +1002,17 @@
       <c r="F8" t="n">
         <v>299</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -995,32 +1021,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Cognac.webp</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1055,14 +1081,17 @@
       <c r="F9" t="n">
         <v>299</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="n">
+        <v>293.02</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -1071,32 +1100,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Mahogany.webp</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1131,14 +1160,17 @@
       <c r="F10" t="n">
         <v>349</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="n">
+        <v>342.02</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -1147,32 +1179,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Blue.webp</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1207,14 +1239,17 @@
       <c r="F11" t="n">
         <v>349</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="n">
+        <v>342.02</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoes using a soft brush or cloth. Ensure the surface is clean and dry.
 2. **Apply the Cream** – Take a small amount on a cloth or applicator brush and spread evenly over the leather in circular motions.
 3. **Let it Dry &amp; Buff** – Allow the cream to absorb for a few minutes, then buff with a clean cloth to achieve a rich shine.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>- Restores original color – Revives faded leather and brings back a rich, even tone
 - Adds long-lasting shine – Delivers a smooth, elegant finish without greasy residue
@@ -1223,32 +1258,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, European Standard, Includes: 1 × Pro Gold Color Shoe Cream, Net Volume: 45 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -Neutral.webp</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>/images/products/Shoe Cream/PRO GOLD  Shoe Cream -White.webp</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1283,7 +1318,10 @@
       <c r="F12" t="n">
         <v>399</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoe or leather surface with a dry cloth.
 2. **Shake the Bottle Well** – Ensures even mixing of the cream and wax ingredients.
@@ -1292,7 +1330,7 @@
 5. **Buff for Extra Shine** – Use a soft cloth or brush to enhance gloss.</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>- Restores original color &amp; shine – Revives faded leather and brings back a rich, polished finish in minutes
 - Deep nourishment &amp; protection – Conditions leather to prevent dryness, cracking, and dullness
@@ -1301,32 +1339,32 @@
 - Built-in sponge applicator – Mess-free and easy application; no extra brush or cloth needed</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, Includes: 1 × Pro Color Shoe Cream with Applicator, Net Volume: 50 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Neutral.webp</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Neutral.webp</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1361,7 +1399,10 @@
       <c r="F13" t="n">
         <v>399</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoe or leather surface with a dry cloth.
 2. **Shake the Bottle Well** – Ensures even mixing of the cream and wax ingredients.
@@ -1370,7 +1411,7 @@
 5. **Buff for Extra Shine** – Use a soft cloth or brush to enhance gloss.</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>- Restores original color &amp; shine – Revives faded leather and brings back a rich, polished finish in minutes
 - Deep nourishment &amp; protection – Conditions leather to prevent dryness, cracking, and dullness
@@ -1379,32 +1420,32 @@
 - Built-in sponge applicator – Mess-free and easy application; no extra brush or cloth needed</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, Includes: 1 × Pro Color Shoe Cream with Applicator, Net Volume: 50 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Neutral.webp</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Black.webp</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1439,7 +1480,10 @@
       <c r="F14" t="n">
         <v>399</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt from the shoe or leather surface with a dry cloth.
 2. **Shake the Bottle Well** – Ensures even mixing of the cream and wax ingredients.
@@ -1448,7 +1492,7 @@
 5. **Buff for Extra Shine** – Use a soft cloth or brush to enhance gloss.</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>- Restores original color &amp; shine – Revives faded leather and brings back a rich, polished finish in minutes
 - Deep nourishment &amp; protection – Conditions leather to prevent dryness, cracking, and dullness
@@ -1457,32 +1501,32 @@
 - Built-in sponge applicator – Mess-free and easy application; no extra brush or cloth needed</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, boots, bags, belts, and accessories</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, Includes: 1 × Pro Color Shoe Cream with Applicator, Net Volume: 50 ml, Product Type: Premium Color Restoring Shoe Cream, Suitable For: Leather and Synthetic Leather shoes, boots, bags, belts, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents, Color Pigments</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>PRO COLOR, Color Refreshing, High Quality, European Experts</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Neutral.webp</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>/images/products/Shoe cream with applicator/Shoe Cream With Applicator -Light Brown.webp</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1517,7 +1561,10 @@
       <c r="F15" t="n">
         <v>249</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" t="n">
+        <v>244.02</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt with a dry cloth.
 2. **Shake Well Before Use** – Ensures even distribution of wax and conditioning agents.
@@ -1526,7 +1573,7 @@
 5. **Ready to Use** – No buffing required; instant self-shine finish achieved.</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>- Self shine – no buffing required – Instant shine formula with polished finish
 - Restores color &amp; shine – Revives dull and faded leather
@@ -1534,32 +1581,32 @@
 - Spill-proof sponge applicator – Smooth, controlled, and mess-free application</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Formula: Wax-Based, Includes: 1 × Self Shine Bottle with Sponge Applicator, Net Volume: 75 ml, Product Type: Self-Shine Liquid Polish, Suitable For: Leather &amp; Synthetic Leather Products, Key Ingredients: Carnauba Wax, Beeswax, Conditioning Agents</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Neutral.webp</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Neutral.webp</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1594,7 +1641,10 @@
       <c r="F16" t="n">
         <v>249</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="n">
+        <v>244.02</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt with a dry cloth.
 2. **Shake Well Before Use** – Ensures even distribution of wax and conditioning agents.
@@ -1603,7 +1653,7 @@
 5. **Ready to Use** – No buffing required; instant self-shine finish achieved.</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>- Self shine – no buffing required – Instant shine formula with polished finish
 - Restores color &amp; shine – Revives dull and faded leather
@@ -1611,32 +1661,32 @@
 - Spill-proof sponge applicator – Smooth, controlled, and mess-free application</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Formula: Wax-Based, Includes: 1 × Self Shine Bottle with Sponge Applicator, Net Volume: 75 ml, Product Type: Self-Shine Liquid Polish, Suitable For: Leather &amp; Synthetic Leather Products, Key Ingredients: Carnauba Wax, Beeswax, Conditioning Agents</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Neutral.webp</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Black.webp</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1671,7 +1721,10 @@
       <c r="F17" t="n">
         <v>249</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="n">
+        <v>244.02</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt with a dry cloth.
 2. **Shake Well Before Use** – Ensures even distribution of wax and conditioning agents.
@@ -1680,7 +1733,7 @@
 5. **Ready to Use** – No buffing required; instant self-shine finish achieved.</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>- Self shine – no buffing required – Instant shine formula with polished finish
 - Restores color &amp; shine – Revives dull and faded leather
@@ -1688,32 +1741,32 @@
 - Spill-proof sponge applicator – Smooth, controlled, and mess-free application</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Formula: Wax-Based, Includes: 1 × Self Shine Bottle with Sponge Applicator, Net Volume: 75 ml, Product Type: Self-Shine Liquid Polish, Suitable For: Leather &amp; Synthetic Leather Products, Key Ingredients: Carnauba Wax, Beeswax, Conditioning Agents</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Neutral.webp</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>/images/products/Self Shine/Self Shine -Brown.webp</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1748,7 +1801,10 @@
       <c r="F18" t="n">
         <v>325</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" t="n">
+        <v>318.5</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt before application.
 2. **Apply Sponge** – Gently press and glide the sponge evenly across the surface.
@@ -1756,7 +1812,7 @@
 4. **Ready to Wear** – No buffing required. Instant shine achieved.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>- Instant &amp; long-lasting shine in seconds – Delivers immediate glossy finish with extended shine
 - Effortless sponge – Built-in sponge allows smooth, quick, and mess-free application
@@ -1765,32 +1821,32 @@
 - 100+ applications – Long-lasting pack for extended usage and value</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic &amp; Eco-Friendly, Formula: Controlled-Flow, Includes: 1 × Quick Shine Sponge, Net Volume: 1 pc, Product Type: Instant Shoe Shine Liquid, Suitable For: Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Neutral.webp</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Neutral.webp</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1825,7 +1881,10 @@
       <c r="F19" t="n">
         <v>325</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" t="n">
+        <v>318.5</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt before application.
 2. **Apply Sponge** – Gently press and glide the sponge evenly across the surface.
@@ -1833,7 +1892,7 @@
 4. **Ready to Wear** – No buffing required. Instant shine achieved.</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>- Instant &amp; long-lasting shine in seconds – Delivers immediate glossy finish with extended shine
 - Effortless sponge – Built-in sponge allows smooth, quick, and mess-free application
@@ -1842,32 +1901,32 @@
 - 100+ applications – Long-lasting pack for extended usage and value</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic &amp; Eco-Friendly, Formula: Controlled-Flow, Includes: 1 × Quick Shine Sponge, Net Volume: 1 pc, Product Type: Instant Shoe Shine Liquid, Suitable For: Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Neutral.webp</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Black.webp</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1902,7 +1961,10 @@
       <c r="F20" t="n">
         <v>325</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="n">
+        <v>318.5</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Remove dust and dirt before application.
 2. **Apply Sponge** – Gently press and glide the sponge evenly across the surface.
@@ -1910,7 +1972,7 @@
 4. **Ready to Wear** – No buffing required. Instant shine achieved.</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>- Instant &amp; long-lasting shine in seconds – Delivers immediate glossy finish with extended shine
 - Effortless sponge – Built-in sponge allows smooth, quick, and mess-free application
@@ -1919,32 +1981,32 @@
 - 100+ applications – Long-lasting pack for extended usage and value</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic &amp; Eco-Friendly, Formula: Controlled-Flow, Includes: 1 × Quick Shine Sponge, Net Volume: 1 pc, Product Type: Instant Shoe Shine Liquid, Suitable For: Leather &amp; Synthetic Leather Products</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>PRO SHINE, Color Refreshing, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Neutral.webp</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>/images/products/Instant Shine/Instant Shiner -Brown.webp</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1979,14 +2041,17 @@
       <c r="F21" t="n">
         <v>425</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="n">
+        <v>416.5</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>1. **Clean the Surface** – Wipe off dust and dirt with a dry or slightly damp cloth. Ensure the surface is clean and dry.
 2. **Apply the Moisturizer** – Apply a small amount using a soft cloth or sponge and spread evenly in gentle circular motions.
 3. **Let it Absorb** – Allow the product to penetrate for a few minutes. Buff lightly with a clean cloth if needed.</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>- Deeply moisturizes leather – Penetrates deep to restore lost moisture and prevent dryness
 - Restores softness &amp; suppleness – Brings stiff, dry leather back to a smooth, flexible feel
@@ -1996,32 +2061,32 @@
 - Safe, water-based formula – Non-toxic and gentle for regular use</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Leather and Synthetic Leather shoes, bags, jackets, belts, furniture, and accessories</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Water-Based, Includes: 1 × Pro Gold Care Leather Moisturizer, Net Volume: 150 ml, Product Type: Leather Conditioning &amp; Moisturizing Cream, Suitable For: Leather and Synthetic Leather shoes, bags, jackets, belts, furniture, and accessories, Key Ingredients: Carnauba Wax, Beeswax, Water-Based Conditioning Agents</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>PRO CARE, Cleaning, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>/images/products/Leather Moisturize -Neutral/Leather Moisturize -Neutral.webp</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>/images/products/Leather Moisturize -Neutral/Leather Moisturize -Neutral.webp</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2056,7 +2121,10 @@
       <c r="F22" t="n">
         <v>399</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>1. **Remove Loose Dirt** – Brush off surface dust and mud before applying.
 2. **Apply Shampoo** – Pump foam directly onto cloth or brush.
@@ -2065,7 +2133,7 @@
 5. **Air Dry** – Let the product dry naturally. Avoid direct heat.</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>- Quick clean, quick dry formula – Advanced fast-acting formula cleans efficiently
 - Instant foam action – Transforms into rich foam that penetrates deep to remove dirt and grime
@@ -2074,32 +2142,32 @@
 - Non-toxic &amp; earth friendly – Eco-conscious formula suitable for regular use</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Sneakers, Colored Leather, Textiles, Canvas, Mesh, Synthetic Materials</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Eco-Friendly, Includes: 1 × Cleaning Shampoo Bottle, Net Volume: 150 ml, Product Type: Cleaning Shampoo, Suitable For: Sneakers, Colored Leather, Textiles, Canvas, Mesh, Synthetic Materials, Key Ingredients: Mild Surfactants, Eco-Friendly Cleaning Agents, Stabilizers</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>/images/products/Power Sneaker Cleaner -Neutral/Power Sneaker Cleaner -Neutral.webp</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>/images/products/Power Sneaker Cleaner -Neutral/Power Sneaker Cleaner -Neutral.webp</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2134,7 +2202,10 @@
       <c r="F23" t="n">
         <v>499</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="n">
+        <v>489.02</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>1. **Remove Loose Dirt** – Brush off dust and mud using the mini brush.
 2. **Apply Shampoo** – Pump foam onto the mini brush.
@@ -2143,7 +2214,7 @@
 5. **Air Dry** – Let dry naturally away from direct heat.</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>- Complete cleaning solution – Everything needed for thorough sneaker cleaning
 - Quick clean &amp; quick dry formula – Fast-acting for efficient results
@@ -2151,32 +2222,32 @@
 - Scratch-resistant mini brush – Compact brush for precise cleaning without surface damage</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Sneakers, Coloured Leather, Textiles, Canvas, Mesh, Synthetic Materials</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Eco-Friendly, Includes: 1 × Cleaning Shampoo (150ml) + 1 × Mini Brush, Net Volume: 150 ml, Product Type: Sneaker Cleaning Kit (Cleaning Shampoo &amp; Mini Brush), Suitable For: Sneakers, Coloured Leather, Textiles, Canvas, Mesh, Synthetic Materials, Key Ingredients: Mild Surfactants, Eco-Friendly Cleaning Agents, Stabilizers</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>/images/products/pro-gold-clean-power-cleaner/1.webp</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>/images/products/pro-gold-clean-power-cleaner/1.webp</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2211,7 +2282,10 @@
       <c r="F24" t="n">
         <v>599</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" t="n">
+        <v>587.02</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>1. **Open the wipe pack** and unfold the wipe.
 2. **Wipe across the surface** of the shoe in gentle circular motions.
@@ -2220,7 +2294,7 @@
 5. **Dispose of wipe** after use.</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>- Pre-moistened cleaning wipes – Ready to use, no water or extra tools needed
 - Instant clean on the go – Convenient for quick cleaning anywhere
@@ -2229,32 +2303,32 @@
 - Pack of 30 – Long-lasting supply for regular use</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Sneakers, Coloured Leather, Textiles, Mesh, Canvas, Synthetic Materials</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Purified Water-Based, Includes: 30 × Sneaker Cleaning Wipes, Net Volume: 30 wipes, Product Type: Sneaker Cleaning Wipes, Suitable For: Sneakers, Coloured Leather, Textiles, Mesh, Canvas, Synthetic Materials, Key Ingredients: Mild Cleaning Agents, Purified Water, Conditioning Additives</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>/images/products/PRO GOLD Clean Sneaker Wipes-Pack of 30 -Neutral/PRO GOLD Clean Sneaker Wipes-Pack of 30 -Neutral.webp</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>/images/products/PRO GOLD Clean Sneaker Wipes-Pack of 30 -Neutral/PRO GOLD Clean Sneaker Wipes-Pack of 30 -Neutral.webp</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2289,26 +2363,29 @@
       <c r="F25" t="n">
         <v>899</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="n">
+        <v>783.02</v>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>Word Doc shared</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2343,7 +2420,10 @@
       <c r="F26" t="n">
         <v>449</v>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" t="n">
+        <v>440.02</v>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>1. **Shake the can well** before use.
 2. **Spray foam evenly** onto the suede or nubuck surface.
@@ -2352,7 +2432,7 @@
 5. **Allow to air dry** naturally. Brush gently once dry to restore nap.</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>- Specialized for suede &amp; nubuck – Formulated specifically for delicate materials
 - Gentle foam action – Deep cleans without causing damage
@@ -2360,32 +2440,32 @@
 - Safe neutral formula – Mild compounds safe for regular use</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Suede &amp; Nubuck Leather</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Neutral Foaming, Includes: 1 × Foam Cleaner Bottle, Net Volume: 150 ml, Product Type: Foam Cleaner, Suitable For: Suede &amp; Nubuck Leather, Key Ingredients: Mild Foaming Agents, Neutral Cleaning Compounds</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>/images/products/Foam Cleaner -Neutral/Foam Cleaner -Neutral.webp</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>/images/products/Foam Cleaner -Neutral/Foam Cleaner -Neutral.webp</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2420,7 +2500,10 @@
       <c r="F27" t="n">
         <v>349</v>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="n">
+        <v>342.02</v>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>1. **Remove insoles** from shoes if possible.
 2. **Hold the spray** 10–15 cm from the shoe opening.
@@ -2429,7 +2512,7 @@
 5. **Use regularly** for continuous freshness.</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>- Eliminates shoe odor – Neutralizes bad smells effectively
 - Long-lasting freshness – Keeps shoes smelling fresh for extended periods
@@ -2438,32 +2521,32 @@
 - Easy spray application – Quick and convenient to use</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Sneakers, Shoes, Canvas, Textiles, Synthetic Materials</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Safety: Non-Toxic, Formula: Spray-Based, Includes: 1 × Shoe Deo Spray Bottle, Net Volume: 150 ml, Product Type: Shoe Deodorizer Spray, Suitable For: Sneakers, Shoes, Canvas, Textiles, Synthetic Materials, Key Ingredients: Deodorizing Agents, Antibacterial Compounds, Fragrance</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>PRO FRESH, Fight Fungi, Long Freshness, European Experts</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>/images/products/Shoe Deo/Shoe Deo.webp</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>/images/products/Shoe Deo/Shoe Deo.webp</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2498,7 +2581,10 @@
       <c r="F28" t="n">
         <v>199</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" t="n">
+        <v>195.02</v>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>1. **Take a Small Amount of Cream** – Dip the brush tip into shoe cream or polish.
 2. **Apply Evenly** – Spread in smooth circular motions across the surface.
@@ -2506,7 +2592,7 @@
 4. **Let It Absorb** – Allow cream to absorb into the leather for a few minutes before buffing.</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>- Even cream application – Ensures uniform spread of shoe cream or polish
 - Round head for precision – Reaches edges, seams, and tight areas
@@ -2514,32 +2600,32 @@
 - Secure &amp; easy grip – Provides control during application</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Shoes, Bags, and Other Leather Articles</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Includes: 1 × Application Brush, Net Content: 1 Piece, Bristle Type: Dense, High-Quality Bristles, Product Type: Shoe Cream Application Brush, Suitable For: Shoes, Bags, and Other Leather Articles, Handle Material: Contoured Beech Wood</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>/images/products/Application Brush/Application Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>/images/products/Application Brush/Application Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2574,7 +2660,10 @@
       <c r="F29" t="n">
         <v>199</v>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" t="n">
+        <v>195.02</v>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>1. **Take a Small Amount of Cream** – Dip the brush tip into shoe cream or polish.
 2. **Apply Evenly** – Spread in smooth circular motions across the surface.
@@ -2582,7 +2671,7 @@
 4. **Let It Absorb** – Allow cream to absorb into the leather for a few minutes before buffing.</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>- Even cream application – Ensures uniform spread of shoe cream or polish
 - Round head for precision – Reaches edges, seams, and tight areas
@@ -2590,32 +2679,32 @@
 - Secure &amp; easy grip – Provides control during application</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Shoes, Bags, and Other Leather Articles</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Includes: 1 × Application Brush, Net Content: 1 Piece, Bristle Type: Dense, High-Quality Bristles, Product Type: Shoe Cream Application Brush, Suitable For: Shoes, Bags, and Other Leather Articles, Handle Material: Contoured Beech Wood</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>/images/products/Application Brush/Application Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>/images/products/Application Brush/Application Brush Light (1).webp</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2650,7 +2739,10 @@
       <c r="F30" t="n">
         <v>399</v>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>1. **Remove Loose Dust** – Brush the surface lightly to remove dust and debris.
 2. **Apply Polish** – Apply shoe cream or polish evenly on the surface.
@@ -2658,7 +2750,7 @@
 4. **Final Finishing** – Continue brushing until the desired shine is achieved.</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>- Excellent shine performance – Dense bristles deliver a rich, glossy shine
 - Effortless dust &amp; dirt removal – Removes dried dust and dirt for a clean finish
@@ -2668,32 +2760,32 @@
 - Professional polishing finish – Smooth, refined, and polished appearance</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>Smooth Leather and Synthetic Shoes, Bags, and Other Articles</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Includes: 1 × Gloss Brush, Net Content: 1 Piece, Bristle Type: Dense, High-Quality Bristles, Product Type: Gloss Brush for Polishing, Suitable For: Smooth Leather and Synthetic Shoes, Bags, and Other Articles, Handle Material: Wooden Body with Deep Grip Groove</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>/images/products/Gloss Brush/Gloss Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>/images/products/Gloss Brush/Gloss Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2728,7 +2820,10 @@
       <c r="F31" t="n">
         <v>399</v>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" t="n">
+        <v>391.02</v>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>1. **Remove Loose Dust** – Brush the surface lightly to remove dust and debris.
 2. **Apply Polish** – Apply shoe cream or polish evenly on the surface.
@@ -2736,7 +2831,7 @@
 4. **Final Finishing** – Continue brushing until the desired shine is achieved.</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>- Excellent shine performance – Dense bristles deliver a rich, glossy shine
 - Effortless dust &amp; dirt removal – Removes dried dust and dirt for a clean finish
@@ -2746,32 +2841,32 @@
 - Professional polishing finish – Smooth, refined, and polished appearance</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>Smooth Leather and Synthetic Shoes, Bags, and Other Articles</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Includes: 1 × Gloss Brush, Net Content: 1 Piece, Bristle Type: Dense, High-Quality Bristles, Product Type: Gloss Brush for Polishing, Suitable For: Smooth Leather and Synthetic Shoes, Bags, and Other Articles, Handle Material: Wooden Body with Deep Grip Groove</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>/images/products/Gloss Brush/Gloss Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>/images/products/Gloss Brush/Gloss Brush Light (1).webp</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2806,7 +2901,10 @@
       <c r="F32" t="n">
         <v>575</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" t="n">
+        <v>563.5</v>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>1. **Remove Surface Dust** – Brush lightly to remove loose dust and debris.
 2. **Apply Shoe Polish** – Apply shoe cream or polish to the surface.
@@ -2814,7 +2912,7 @@
 4. **Final Finishing Shine** – Continue buffing until the desired gloss is achieved.</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>- Premium 100% genuine horse hair bristles – Dense and soft for superior polishing
 - Silky high gloss finish – Delivers a rich, glossy shine on polished surfaces
@@ -2822,32 +2920,32 @@
 - Ergonomic curved design – Comfortable grip for effortless buffing</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>Shoes, Bags, and Other Leather Articles</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Includes: 1 × Horse Hair Polishing Brush, Net Content: 1 Piece, Bristle Type: 100% Genuine Horse Hair (Dense &amp; Soft), Product Type: Horse Hair Shoe Polishing Brush, Suitable For: Shoes, Bags, and Other Leather Articles, Handle Material: Contoured Beech Wood</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>/images/products/Horse hair Brush/Horse Hair Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>/images/products/Horse hair Brush/Horse Hair Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2882,7 +2980,10 @@
       <c r="F33" t="n">
         <v>575</v>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" t="n">
+        <v>563.5</v>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>1. **Remove Surface Dust** – Brush lightly to remove loose dust and debris.
 2. **Apply Shoe Polish** – Apply shoe cream or polish to the surface.
@@ -2890,7 +2991,7 @@
 4. **Final Finishing Shine** – Continue buffing until the desired gloss is achieved.</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>- Premium 100% genuine horse hair bristles – Dense and soft for superior polishing
 - Silky high gloss finish – Delivers a rich, glossy shine on polished surfaces
@@ -2898,32 +2999,32 @@
 - Ergonomic curved design – Comfortable grip for effortless buffing</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>Shoes, Bags, and Other Leather Articles</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Includes: 1 × Horse Hair Polishing Brush, Net Content: 1 Piece, Bristle Type: 100% Genuine Horse Hair (Dense &amp; Soft), Product Type: Horse Hair Shoe Polishing Brush, Suitable For: Shoes, Bags, and Other Leather Articles, Handle Material: Contoured Beech Wood</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>/images/products/Horse hair Brush/Horse Hair Brush Dark (1).webp</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>/images/products/Horse hair Brush/Horse Hair Brush Light (1).webp</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2958,7 +3059,10 @@
       <c r="F34" t="n">
         <v>250</v>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" t="n">
+        <v>245</v>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>1. **Dry Brushing** – Gently brush the surface to remove loose dust and dirt.
 2. **Remove Embedded Dirt** – Use firmer strokes to lift ingrained particles.
@@ -2966,7 +3070,7 @@
 4. **Clean Edges &amp; Welts** – Use brush edges to clean sole edges and welt areas.</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>- Specially designed for suede &amp; nubuck – Engineered to clean delicate materials safely
 - Removes dust &amp; ingrained dirt – Effectively lifts dust, dirt, and embedded particles
@@ -2974,32 +3078,32 @@
 - Cleans sole edge &amp; welt – Efficiently cleans hard-to-reach areas</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Suede and Nubuck Shoes, Bags, and Other Articles</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Includes: 1 × Suede Brush, Net Content: 1 Piece, Bristle Type: Dual Bristles for Cleaning &amp; Nap Restoration, Product Type: Suede &amp; Nubuck Cleaning Brush, Suitable For: Suede and Nubuck Shoes, Bags, and Other Articles</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>/images/products/Suede Brush/Suede Brush Rubber Black (1).webp</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>/images/products/Suede Brush/Suede Brush Rubber Black (1).webp</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3034,7 +3138,10 @@
       <c r="F35" t="n">
         <v>3999</v>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" t="n">
+        <v>3199.2</v>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>1. **Remove the shoe tree** from the packaging.
 2. **Insert into shoes** immediately after taking them off.
@@ -3043,7 +3150,7 @@
 5. **Use regularly** for best shape retention and freshness.</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>- 100% natural cedar wood – High-quality natural cedar for superior shoe care
 - Maintains original shape – Gently stretches and supports the shoe to retain its structure
@@ -3052,28 +3159,28 @@
 - Natural fresh fragrance – Cedar wood aroma keeps shoes smelling fresh</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
         <is>
           <t>Usage: Suitable for all types of shoes, Function: Shape retention, moisture absorption, and freshness, Includes: 1 Pair of Shoe Trees, Material: 100% Natural Cedar Wood, Fragrance: Natural cedar wood aroma, Net Content: 1 Pair, Product Type: Cedar Wood Shoe Tree</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3108,7 +3215,10 @@
       <c r="F36" t="n">
         <v>3999</v>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" t="n">
+        <v>3199.2</v>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>1. **Remove the shoe tree** from the packaging.
 2. **Insert into shoes** immediately after taking them off.
@@ -3117,7 +3227,7 @@
 5. **Use regularly** for best shape retention and freshness.</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>- 100% natural cedar wood – High-quality natural cedar for superior shoe care
 - Maintains original shape – Gently stretches and supports the shoe to retain its structure
@@ -3126,28 +3236,28 @@
 - Natural fresh fragrance – Cedar wood aroma keeps shoes smelling fresh</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
         <is>
           <t>Usage: Suitable for all types of shoes, Function: Shape retention, moisture absorption, and freshness, Includes: 1 Pair of Shoe Trees, Material: 100% Natural Cedar Wood, Fragrance: Natural cedar wood aroma, Net Content: 1 Pair, Product Type: Cedar Wood Shoe Tree</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3182,7 +3292,10 @@
       <c r="F37" t="n">
         <v>3999</v>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" t="n">
+        <v>3199.2</v>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>1. **Remove the shoe tree** from the packaging.
 2. **Insert into shoes** immediately after taking them off.
@@ -3191,7 +3304,7 @@
 5. **Use regularly** for best shape retention and freshness.</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>- 100% natural cedar wood – High-quality natural cedar for superior shoe care
 - Maintains original shape – Gently stretches and supports the shoe to retain its structure
@@ -3200,28 +3313,28 @@
 - Natural fresh fragrance – Cedar wood aroma keeps shoes smelling fresh</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
         <is>
           <t>Usage: Suitable for all types of shoes, Function: Shape retention, moisture absorption, and freshness, Includes: 1 Pair of Shoe Trees, Material: 100% Natural Cedar Wood, Fragrance: Natural cedar wood aroma, Net Content: 1 Pair, Product Type: Cedar Wood Shoe Tree</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3256,7 +3369,10 @@
       <c r="F38" t="n">
         <v>3999</v>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" t="n">
+        <v>3199.2</v>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>1. **Remove the shoe tree** from the packaging.
 2. **Insert into shoes** immediately after taking them off.
@@ -3265,7 +3381,7 @@
 5. **Use regularly** for best shape retention and freshness.</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>- 100% natural cedar wood – High-quality natural cedar for superior shoe care
 - Maintains original shape – Gently stretches and supports the shoe to retain its structure
@@ -3274,28 +3390,28 @@
 - Natural fresh fragrance – Cedar wood aroma keeps shoes smelling fresh</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
         <is>
           <t>Usage: Suitable for all types of shoes, Function: Shape retention, moisture absorption, and freshness, Includes: 1 Pair of Shoe Trees, Material: 100% Natural Cedar Wood, Fragrance: Natural cedar wood aroma, Net Content: 1 Pair, Product Type: Cedar Wood Shoe Tree</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3330,7 +3446,10 @@
       <c r="F39" t="n">
         <v>3999</v>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" t="n">
+        <v>3199.2</v>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>1. **Remove the shoe tree** from the packaging.
 2. **Insert into shoes** immediately after taking them off.
@@ -3339,7 +3458,7 @@
 5. **Use regularly** for best shape retention and freshness.</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>- 100% natural cedar wood – High-quality natural cedar for superior shoe care
 - Maintains original shape – Gently stretches and supports the shoe to retain its structure
@@ -3348,28 +3467,28 @@
 - Natural fresh fragrance – Cedar wood aroma keeps shoes smelling fresh</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
         <is>
           <t>Usage: Suitable for all types of shoes, Function: Shape retention, moisture absorption, and freshness, Includes: 1 Pair of Shoe Trees, Material: 100% Natural Cedar Wood, Fragrance: Natural cedar wood aroma, Net Content: 1 Pair, Product Type: Cedar Wood Shoe Tree</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Premium Shoe Tree (1).webp</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3404,30 +3523,33 @@
       <c r="F40" t="n">
         <v>899</v>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" t="n">
+        <v>699</v>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>Word Doc shared</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3462,30 +3584,33 @@
       <c r="F41" t="n">
         <v>899</v>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" t="n">
+        <v>699</v>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>Word Doc shared</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3520,30 +3645,33 @@
       <c r="F42" t="n">
         <v>899</v>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" t="n">
+        <v>699</v>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>Word Doc shared</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>/images/products/Shoe Tree/Shoe Tree With Spiral.webp</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3578,7 +3706,10 @@
       <c r="F43" t="n">
         <v>325</v>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" t="n">
+        <v>318.5</v>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>1. **Remove Surface Dust** – Use sponge side gently to remove loose dirt and dust.
 2. **Erase Stubborn Marks** – Rub the gum eraser lightly on stains, scuffs, or marks.
@@ -3586,7 +3717,7 @@
 4. **Regular Maintenance** – Use regularly to maintain cleanliness and appearance.</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>- Innovative 2-in-1 design – Combines cleaning sponge and gum eraser for complete care
 - Ideal for daily maintenance – Perfect for regular upkeep of suede and nubuck items
@@ -3595,32 +3726,32 @@
 - Works on all colors – Safe for all suede and nubuck shades</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Suede and Nubuck Shoes, Boots, and Bags</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Includes: 1 × Suede 2in1 Sponge &amp; Eraser, Material: Cleaning Sponge + Gum Eraser, Net Content: 1 Piece, Product Type: 2-in-1 Suede Cleaning Sponge &amp; Eraser, Suitable For: Suede and Nubuck Shoes, Boots, and Bags, Color Compatibility: Works on all colors of suede and nubuck</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>/images/products/Nubuck 2 in 1 Neutral/Nubuck 2 in 1 Neutral (1).webp</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>/images/products/Nubuck 2 in 1 Neutral/Nubuck 2 in 1 Neutral (1).webp</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3655,30 +3786,33 @@
       <c r="F44" t="n">
         <v>249</v>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" t="n">
+        <v>244.02</v>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>Word Doc shared</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
         <is>
           <t>PRO CLEAN, Cleaning, Effective Clean, European Experts</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>/images/products/Perfect Clean Gel 50ml Neutral/Perfect Clean Gel 50ml Neutral (1).webp</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>/images/products/Perfect Clean Gel 50ml Neutral/Perfect Clean Gel 50ml Neutral (1).webp</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3713,7 +3847,10 @@
       <c r="F45" t="n">
         <v>549</v>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" t="n">
+        <v>538.02</v>
+      </c>
+      <c r="H45" t="inlineStr">
         <is>
           <t>1. **Remove dust and dirt** from the suede or nubuck using a brush.
 2. **Shake the spray** before use.
@@ -3722,7 +3859,7 @@
 5. **Once dry, brush gently** to restore the suede nap.</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>- Renovates &amp; restores – Revives suede &amp; nubuck colors while conditioning leather
 - Dirt &amp; water repellent – Creates a protective layer that repels moisture and dirt
@@ -3730,32 +3867,32 @@
 - Multi-use care – Suitable for suede &amp; nubuck shoes, bags, and jackets</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Suede &amp; Nubuck Leather – Shoes, Bags &amp; Jackets</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Color: Neutral (Colorless), Formula: Water-Based, European Standard, Features: Restores Color, Conditions Leather, Water &amp; Dirt Repellent, Includes: 1 × Suede &amp; Nubuck Renovator Spray, Net Volume: 180 ml, Product Type: Suede &amp; Nubuck Renovator Spray, Suitable For: Suede &amp; Nubuck Leather – Shoes, Bags &amp; Jackets</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>PRO CARE, Cleaning, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>/images/products/Suede N Nubuck Spray 180 ml-Neutral/Suede N Nubuck Spray 180 ml-Neutral 1.webp</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>/images/products/Suede N Nubuck Spray 180 ml-Neutral/Suede N Nubuck Spray 180 ml-Neutral 1.webp</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3790,7 +3927,10 @@
       <c r="F46" t="n">
         <v>599</v>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" t="n">
+        <v>587.02</v>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>1. **Ensure the shoes are clean and completely dry** before application.
 2. **Shake the spray bottle well.**
@@ -3800,7 +3940,7 @@
 6. **For enhanced water resistance** – Apply two additional coats after drying.</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>- Ultimate shoe protection – Shields footwear from dirt, water, snow, and stains
 - Advanced nano-technology formula – Creates an invisible, breathable protective layer
@@ -3809,32 +3949,32 @@
 - Maintains original look – Transparent coating preserves the natural finish</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>Suede, Nubuck, Leather, Canvas, Fabric, and Sports Shoes; Bags, jackets, and fabric accessories</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Function: Water repellency, stain protection, and dirt resistance, Includes: 1 × Hydroshield Spray Bottle, Net Volume: 180 ml, Product Type: Water &amp; Stain Protector Spray, Suitable For: Suede, Nubuck, Leather, Canvas, Fabric, and Sports Shoes; Bags, jackets, and fabric accessories</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>PRO CARE, Cleaning, Shine, European Experts</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>/images/products/New folder (2)/Hydroshield 180 ml-Neutral (1).webp</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>/images/products/New folder (2)/Hydroshield 180 ml-Neutral (1).webp</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3869,22 +4009,25 @@
       <c r="F47" t="n">
         <v>649</v>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="G47" t="n">
+        <v>599</v>
+      </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr">
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3919,14 +4062,17 @@
       <c r="F48" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G48" s="1" t="inlineStr">
+      <c r="G48" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H48" s="1" t="inlineStr">
+      <c r="I48" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -3935,28 +4081,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I48" s="1" t="inlineStr">
+      <c r="J48" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J48" s="1" t="inlineStr">
+      <c r="K48" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K48" s="1" t="inlineStr">
+      <c r="L48" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L48" s="1" t="inlineStr">
+      <c r="M48" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M48" s="1" t="inlineStr"/>
-      <c r="N48" s="1" t="inlineStr">
+      <c r="N48" s="1" t="inlineStr"/>
+      <c r="O48" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3991,14 +4137,17 @@
       <c r="F49" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G49" s="1" t="inlineStr">
+      <c r="G49" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H49" s="1" t="inlineStr">
+      <c r="I49" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -4007,28 +4156,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I49" s="1" t="inlineStr">
+      <c r="J49" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J49" s="1" t="inlineStr">
+      <c r="K49" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K49" s="1" t="inlineStr">
+      <c r="L49" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L49" s="1" t="inlineStr">
+      <c r="M49" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M49" s="1" t="inlineStr"/>
-      <c r="N49" s="1" t="inlineStr">
+      <c r="N49" s="1" t="inlineStr"/>
+      <c r="O49" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4063,14 +4212,17 @@
       <c r="F50" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G50" s="1" t="inlineStr">
+      <c r="G50" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H50" s="1" t="inlineStr">
+      <c r="I50" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -4079,28 +4231,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I50" s="1" t="inlineStr">
+      <c r="J50" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J50" s="1" t="inlineStr">
+      <c r="K50" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K50" s="1" t="inlineStr">
+      <c r="L50" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L50" s="1" t="inlineStr">
+      <c r="M50" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M50" s="1" t="inlineStr"/>
-      <c r="N50" s="1" t="inlineStr">
+      <c r="N50" s="1" t="inlineStr"/>
+      <c r="O50" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4135,14 +4287,17 @@
       <c r="F51" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G51" s="1" t="inlineStr">
+      <c r="G51" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H51" s="1" t="inlineStr">
+      <c r="I51" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -4151,28 +4306,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I51" s="1" t="inlineStr">
+      <c r="J51" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J51" s="1" t="inlineStr">
+      <c r="K51" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K51" s="1" t="inlineStr">
+      <c r="L51" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L51" s="1" t="inlineStr">
+      <c r="M51" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M51" s="1" t="inlineStr"/>
-      <c r="N51" s="1" t="inlineStr">
+      <c r="N51" s="1" t="inlineStr"/>
+      <c r="O51" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4207,14 +4362,17 @@
       <c r="F52" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G52" s="1" t="inlineStr">
+      <c r="G52" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H52" s="1" t="inlineStr">
+      <c r="I52" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -4223,28 +4381,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I52" s="1" t="inlineStr">
+      <c r="J52" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J52" s="1" t="inlineStr">
+      <c r="K52" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K52" s="1" t="inlineStr">
+      <c r="L52" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L52" s="1" t="inlineStr">
+      <c r="M52" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M52" s="1" t="inlineStr"/>
-      <c r="N52" s="1" t="inlineStr">
+      <c r="N52" s="1" t="inlineStr"/>
+      <c r="O52" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4279,14 +4437,17 @@
       <c r="F53" s="1" t="n">
         <v>699</v>
       </c>
-      <c r="G53" s="1" t="inlineStr">
+      <c r="G53" s="1" t="n">
+        <v>685.02</v>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Memory Foam Insoles into your shoes with the fabric side facing up.
 2. **Ensure** the insole fits flat and properly inside the shoe.
 3. **Use daily** for enhanced comfort and pressure relief.</t>
         </is>
       </c>
-      <c r="H53" s="1" t="inlineStr">
+      <c r="I53" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort – Soft memory foam cushioning for superior daily comfort
 - Versatile use – Perfect for both formal and casual shoes; unisex design
@@ -4295,28 +4456,28 @@
 - Breathable &amp; comfortable – Enhances comfort during long hours of standing or walking</t>
         </is>
       </c>
-      <c r="I53" s="1" t="inlineStr">
+      <c r="J53" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J53" s="1" t="inlineStr">
+      <c r="K53" s="1" t="inlineStr">
         <is>
           <t>Design: Unisex, cushioned comfort insole, Function: Comfort, pressure relief, and fatigue reduction, Includes: 1 Pair of Memory Foam Insoles, Material: High-Quality Memory Foam, Net Content: 1 Pair, Product Type: Memory Foam Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K53" s="1" t="inlineStr">
+      <c r="L53" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L53" s="1" t="inlineStr">
+      <c r="M53" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M53" s="1" t="inlineStr"/>
-      <c r="N53" s="1" t="inlineStr">
+      <c r="N53" s="1" t="inlineStr"/>
+      <c r="O53" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4351,7 +4512,10 @@
       <c r="F54" s="1" t="n">
         <v>225</v>
       </c>
-      <c r="G54" s="1" t="inlineStr">
+      <c r="G54" s="1" t="n">
+        <v>220.5</v>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
         <is>
           <t>1. **Align** the old insole with the new PRO Insole.
 2. **Trace** the outline where the new insole overlaps.
@@ -4359,7 +4523,7 @@
 4. **Insert** the trimmed insoles into your shoes with the fabric side facing up.</t>
         </is>
       </c>
-      <c r="H54" s="1" t="inlineStr">
+      <c r="I54" s="1" t="inlineStr">
         <is>
           <t>- 3-layer comfort design – Viscous top layer and two layers of pure latex foam
 - Excellent walking comfort – Soft cushioned insoles for enhanced daily comfort
@@ -4368,28 +4532,28 @@
 - Lightweight &amp; flexible – Ensures natural movement without adding bulk</t>
         </is>
       </c>
-      <c r="I54" s="1" t="inlineStr">
+      <c r="J54" s="1" t="inlineStr">
         <is>
           <t>Formal and casual shoes</t>
         </is>
       </c>
-      <c r="J54" s="1" t="inlineStr">
+      <c r="K54" s="1" t="inlineStr">
         <is>
           <t>Function: Comfort, cushioning, ventilation, and odor control, Includes: 1 Pair of 3-Layer Insoles, Material: Viscous Top Layer + Dual Pure Latex Foam Layers, Net Content: 1 Pair, Product Type: 3-Layer Cushion Insoles, Suitable For: Formal and casual shoes</t>
         </is>
       </c>
-      <c r="K54" s="1" t="inlineStr">
+      <c r="L54" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L54" s="1" t="inlineStr">
+      <c r="M54" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M54" s="1" t="inlineStr"/>
-      <c r="N54" s="1" t="inlineStr">
+      <c r="N54" s="1" t="inlineStr"/>
+      <c r="O54" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4424,7 +4588,10 @@
       <c r="F55" s="1" t="n">
         <v>549</v>
       </c>
-      <c r="G55" s="1" t="inlineStr">
+      <c r="G55" s="1" t="n">
+        <v>538.02</v>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Comfort Gel Insoles into your shoes with the fabric side facing up.
 2. **Adjust** to ensure the insoles lie flat inside the shoes.
@@ -4432,7 +4599,7 @@
 4. **Use daily** for enhanced comfort, shock absorption, and moisture control.</t>
         </is>
       </c>
-      <c r="H55" s="1" t="inlineStr">
+      <c r="I55" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort &amp; support – Soft gel cushioning for everyday wear
 - Superior shock absorption – Minimizes impact on feet and joints for smoother walking
@@ -4441,28 +4608,28 @@
 - Pressure relief – Distributes foot pressure evenly for improved comfort</t>
         </is>
       </c>
-      <c r="I55" s="1" t="inlineStr">
+      <c r="J55" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J55" s="1" t="inlineStr">
+      <c r="K55" s="1" t="inlineStr">
         <is>
           <t>Design: Cushioned, moisture-wicking, shock-absorbing insole, Function: Comfort, shock absorption, moisture control, and support, Includes: 1 Pair of Gel Insoles, Material: High-Quality Gel, Net Content: 1 Pair, Product Type: Gel Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K55" s="1" t="inlineStr">
+      <c r="L55" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L55" s="1" t="inlineStr">
+      <c r="M55" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M55" s="1" t="inlineStr"/>
-      <c r="N55" s="1" t="inlineStr">
+      <c r="N55" s="1" t="inlineStr"/>
+      <c r="O55" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4497,7 +4664,10 @@
       <c r="F56" s="1" t="n">
         <v>549</v>
       </c>
-      <c r="G56" s="1" t="inlineStr">
+      <c r="G56" s="1" t="n">
+        <v>538.02</v>
+      </c>
+      <c r="H56" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the PRO Comfort Gel Insoles into your shoes with the fabric side facing up.
 2. **Adjust** to ensure the insoles lie flat inside the shoes.
@@ -4505,7 +4675,7 @@
 4. **Use daily** for enhanced comfort, shock absorption, and moisture control.</t>
         </is>
       </c>
-      <c r="H56" s="1" t="inlineStr">
+      <c r="I56" s="1" t="inlineStr">
         <is>
           <t>- All-day comfort &amp; support – Soft gel cushioning for everyday wear
 - Superior shock absorption – Minimizes impact on feet and joints for smoother walking
@@ -4514,28 +4684,28 @@
 - Pressure relief – Distributes foot pressure evenly for improved comfort</t>
         </is>
       </c>
-      <c r="I56" s="1" t="inlineStr">
+      <c r="J56" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J56" s="1" t="inlineStr">
+      <c r="K56" s="1" t="inlineStr">
         <is>
           <t>Design: Cushioned, moisture-wicking, shock-absorbing insole, Function: Comfort, shock absorption, moisture control, and support, Includes: 1 Pair of Gel Insoles, Material: High-Quality Gel, Net Content: 1 Pair, Product Type: Gel Insoles, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K56" s="1" t="inlineStr">
+      <c r="L56" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L56" s="1" t="inlineStr">
+      <c r="M56" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M56" s="1" t="inlineStr"/>
-      <c r="N56" s="1" t="inlineStr">
+      <c r="N56" s="1" t="inlineStr"/>
+      <c r="O56" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4570,7 +4740,10 @@
       <c r="F57" s="1" t="n">
         <v>649</v>
       </c>
-      <c r="G57" s="1" t="inlineStr">
+      <c r="G57" s="1" t="n">
+        <v>636.02</v>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the Air Walk Gel Insoles into your shoes with the fabric side facing up.
 2. **Adjust** to ensure they lie flat inside the shoe.
@@ -4578,7 +4751,7 @@
 4. **Use daily** for enhanced comfort and shock absorption.</t>
         </is>
       </c>
-      <c r="H57" s="1" t="inlineStr">
+      <c r="I57" s="1" t="inlineStr">
         <is>
           <t>- Enhanced all-day comfort – Soft gel cushioning with every step
 - Superior shock absorption – Minimizes impact on feet and joints
@@ -4587,28 +4760,28 @@
 - Moisture-wicking – Helps keep feet dry and reduces discomfort</t>
         </is>
       </c>
-      <c r="I57" s="1" t="inlineStr">
+      <c r="J57" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J57" s="1" t="inlineStr">
+      <c r="K57" s="1" t="inlineStr">
         <is>
           <t>Design: Anti-slip, shock-absorbing cushioned insole, Function: Comfort, shock absorption, and stability, Includes: 1 Pair of Air Walk Gel Insoles, Material: High-Quality Gel with Air Cushion, Net Content: 1 Pair, Product Type: Gel Insoles with Air Cushion Technology, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K57" s="1" t="inlineStr">
+      <c r="L57" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L57" s="1" t="inlineStr">
+      <c r="M57" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M57" s="1" t="inlineStr"/>
-      <c r="N57" s="1" t="inlineStr">
+      <c r="N57" s="1" t="inlineStr"/>
+      <c r="O57" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4643,7 +4816,10 @@
       <c r="F58" s="1" t="n">
         <v>649</v>
       </c>
-      <c r="G58" s="1" t="inlineStr">
+      <c r="G58" s="1" t="n">
+        <v>636.02</v>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
         <is>
           <t>1. **Insert** the Air Walk Gel Insoles into your shoes with the fabric side facing up.
 2. **Adjust** to ensure they lie flat inside the shoe.
@@ -4651,7 +4827,7 @@
 4. **Use daily** for enhanced comfort and shock absorption.</t>
         </is>
       </c>
-      <c r="H58" s="1" t="inlineStr">
+      <c r="I58" s="1" t="inlineStr">
         <is>
           <t>- Enhanced all-day comfort – Soft gel cushioning with every step
 - Superior shock absorption – Minimizes impact on feet and joints
@@ -4660,28 +4836,28 @@
 - Moisture-wicking – Helps keep feet dry and reduces discomfort</t>
         </is>
       </c>
-      <c r="I58" s="1" t="inlineStr">
+      <c r="J58" s="1" t="inlineStr">
         <is>
           <t>Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="J58" s="1" t="inlineStr">
+      <c r="K58" s="1" t="inlineStr">
         <is>
           <t>Design: Anti-slip, shock-absorbing cushioned insole, Function: Comfort, shock absorption, and stability, Includes: 1 Pair of Air Walk Gel Insoles, Material: High-Quality Gel with Air Cushion, Net Content: 1 Pair, Product Type: Gel Insoles with Air Cushion Technology, Suitable For: Formal shoes, casual shoes, and sneakers</t>
         </is>
       </c>
-      <c r="K58" s="1" t="inlineStr">
+      <c r="L58" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L58" s="1" t="inlineStr">
+      <c r="M58" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M58" s="1" t="inlineStr"/>
-      <c r="N58" s="1" t="inlineStr">
+      <c r="N58" s="1" t="inlineStr"/>
+      <c r="O58" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4716,22 +4892,25 @@
       <c r="F59" s="1" t="n">
         <v>249</v>
       </c>
-      <c r="G59" s="1" t="inlineStr"/>
+      <c r="G59" s="1" t="n">
+        <v>244.02</v>
+      </c>
       <c r="H59" s="1" t="inlineStr"/>
       <c r="I59" s="1" t="inlineStr"/>
       <c r="J59" s="1" t="inlineStr"/>
-      <c r="K59" s="1" t="inlineStr">
+      <c r="K59" s="1" t="inlineStr"/>
+      <c r="L59" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L59" s="1" t="inlineStr">
+      <c r="M59" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M59" s="1" t="inlineStr"/>
-      <c r="N59" s="1" t="inlineStr">
+      <c r="N59" s="1" t="inlineStr"/>
+      <c r="O59" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4766,22 +4945,25 @@
       <c r="F60" s="1" t="n">
         <v>249</v>
       </c>
-      <c r="G60" s="1" t="inlineStr"/>
+      <c r="G60" s="1" t="n">
+        <v>244.02</v>
+      </c>
       <c r="H60" s="1" t="inlineStr"/>
       <c r="I60" s="1" t="inlineStr"/>
       <c r="J60" s="1" t="inlineStr"/>
-      <c r="K60" s="1" t="inlineStr">
+      <c r="K60" s="1" t="inlineStr"/>
+      <c r="L60" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L60" s="1" t="inlineStr">
+      <c r="M60" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M60" s="1" t="inlineStr"/>
-      <c r="N60" s="1" t="inlineStr">
+      <c r="N60" s="1" t="inlineStr"/>
+      <c r="O60" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4816,22 +4998,25 @@
       <c r="F61" s="1" t="n">
         <v>299</v>
       </c>
-      <c r="G61" s="1" t="inlineStr"/>
+      <c r="G61" s="1" t="n">
+        <v>299</v>
+      </c>
       <c r="H61" s="1" t="inlineStr"/>
       <c r="I61" s="1" t="inlineStr"/>
       <c r="J61" s="1" t="inlineStr"/>
-      <c r="K61" s="1" t="inlineStr">
+      <c r="K61" s="1" t="inlineStr"/>
+      <c r="L61" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L61" s="1" t="inlineStr">
+      <c r="M61" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M61" s="1" t="inlineStr"/>
-      <c r="N61" s="1" t="inlineStr">
+      <c r="N61" s="1" t="inlineStr"/>
+      <c r="O61" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4866,22 +5051,25 @@
       <c r="F62" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G62" s="1" t="inlineStr"/>
+      <c r="G62" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H62" s="1" t="inlineStr"/>
       <c r="I62" s="1" t="inlineStr"/>
       <c r="J62" s="1" t="inlineStr"/>
-      <c r="K62" s="1" t="inlineStr">
+      <c r="K62" s="1" t="inlineStr"/>
+      <c r="L62" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L62" s="1" t="inlineStr">
+      <c r="M62" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M62" s="1" t="inlineStr"/>
-      <c r="N62" s="1" t="inlineStr">
+      <c r="N62" s="1" t="inlineStr"/>
+      <c r="O62" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4916,22 +5104,25 @@
       <c r="F63" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G63" s="1" t="inlineStr"/>
+      <c r="G63" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H63" s="1" t="inlineStr"/>
       <c r="I63" s="1" t="inlineStr"/>
       <c r="J63" s="1" t="inlineStr"/>
-      <c r="K63" s="1" t="inlineStr">
+      <c r="K63" s="1" t="inlineStr"/>
+      <c r="L63" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L63" s="1" t="inlineStr">
+      <c r="M63" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M63" s="1" t="inlineStr"/>
-      <c r="N63" s="1" t="inlineStr">
+      <c r="N63" s="1" t="inlineStr"/>
+      <c r="O63" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4966,22 +5157,25 @@
       <c r="F64" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G64" s="1" t="inlineStr"/>
+      <c r="G64" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H64" s="1" t="inlineStr"/>
       <c r="I64" s="1" t="inlineStr"/>
       <c r="J64" s="1" t="inlineStr"/>
-      <c r="K64" s="1" t="inlineStr">
+      <c r="K64" s="1" t="inlineStr"/>
+      <c r="L64" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L64" s="1" t="inlineStr">
+      <c r="M64" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M64" s="1" t="inlineStr"/>
-      <c r="N64" s="1" t="inlineStr">
+      <c r="N64" s="1" t="inlineStr"/>
+      <c r="O64" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5016,22 +5210,25 @@
       <c r="F65" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G65" s="1" t="inlineStr"/>
+      <c r="G65" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H65" s="1" t="inlineStr"/>
       <c r="I65" s="1" t="inlineStr"/>
       <c r="J65" s="1" t="inlineStr"/>
-      <c r="K65" s="1" t="inlineStr">
+      <c r="K65" s="1" t="inlineStr"/>
+      <c r="L65" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L65" s="1" t="inlineStr">
+      <c r="M65" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M65" s="1" t="inlineStr"/>
-      <c r="N65" s="1" t="inlineStr">
+      <c r="N65" s="1" t="inlineStr"/>
+      <c r="O65" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5066,22 +5263,25 @@
       <c r="F66" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G66" s="1" t="inlineStr"/>
+      <c r="G66" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H66" s="1" t="inlineStr"/>
       <c r="I66" s="1" t="inlineStr"/>
       <c r="J66" s="1" t="inlineStr"/>
-      <c r="K66" s="1" t="inlineStr">
+      <c r="K66" s="1" t="inlineStr"/>
+      <c r="L66" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L66" s="1" t="inlineStr">
+      <c r="M66" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M66" s="1" t="inlineStr"/>
-      <c r="N66" s="1" t="inlineStr">
+      <c r="N66" s="1" t="inlineStr"/>
+      <c r="O66" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5116,22 +5316,25 @@
       <c r="F67" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G67" s="1" t="inlineStr"/>
+      <c r="G67" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H67" s="1" t="inlineStr"/>
       <c r="I67" s="1" t="inlineStr"/>
       <c r="J67" s="1" t="inlineStr"/>
-      <c r="K67" s="1" t="inlineStr">
+      <c r="K67" s="1" t="inlineStr"/>
+      <c r="L67" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L67" s="1" t="inlineStr">
+      <c r="M67" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M67" s="1" t="inlineStr"/>
-      <c r="N67" s="1" t="inlineStr">
+      <c r="N67" s="1" t="inlineStr"/>
+      <c r="O67" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5166,22 +5369,25 @@
       <c r="F68" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G68" s="1" t="inlineStr"/>
+      <c r="G68" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H68" s="1" t="inlineStr"/>
       <c r="I68" s="1" t="inlineStr"/>
       <c r="J68" s="1" t="inlineStr"/>
-      <c r="K68" s="1" t="inlineStr">
+      <c r="K68" s="1" t="inlineStr"/>
+      <c r="L68" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L68" s="1" t="inlineStr">
+      <c r="M68" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M68" s="1" t="inlineStr"/>
-      <c r="N68" s="1" t="inlineStr">
+      <c r="N68" s="1" t="inlineStr"/>
+      <c r="O68" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5216,22 +5422,25 @@
       <c r="F69" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G69" s="1" t="inlineStr"/>
+      <c r="G69" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H69" s="1" t="inlineStr"/>
       <c r="I69" s="1" t="inlineStr"/>
       <c r="J69" s="1" t="inlineStr"/>
-      <c r="K69" s="1" t="inlineStr">
+      <c r="K69" s="1" t="inlineStr"/>
+      <c r="L69" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L69" s="1" t="inlineStr">
+      <c r="M69" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M69" s="1" t="inlineStr"/>
-      <c r="N69" s="1" t="inlineStr">
+      <c r="N69" s="1" t="inlineStr"/>
+      <c r="O69" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5266,22 +5475,25 @@
       <c r="F70" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G70" s="1" t="inlineStr"/>
+      <c r="G70" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H70" s="1" t="inlineStr"/>
       <c r="I70" s="1" t="inlineStr"/>
       <c r="J70" s="1" t="inlineStr"/>
-      <c r="K70" s="1" t="inlineStr">
+      <c r="K70" s="1" t="inlineStr"/>
+      <c r="L70" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L70" s="1" t="inlineStr">
+      <c r="M70" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M70" s="1" t="inlineStr"/>
-      <c r="N70" s="1" t="inlineStr">
+      <c r="N70" s="1" t="inlineStr"/>
+      <c r="O70" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5316,22 +5528,25 @@
       <c r="F71" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G71" s="1" t="inlineStr"/>
+      <c r="G71" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H71" s="1" t="inlineStr"/>
       <c r="I71" s="1" t="inlineStr"/>
       <c r="J71" s="1" t="inlineStr"/>
-      <c r="K71" s="1" t="inlineStr">
+      <c r="K71" s="1" t="inlineStr"/>
+      <c r="L71" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L71" s="1" t="inlineStr">
+      <c r="M71" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M71" s="1" t="inlineStr"/>
-      <c r="N71" s="1" t="inlineStr">
+      <c r="N71" s="1" t="inlineStr"/>
+      <c r="O71" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5366,22 +5581,25 @@
       <c r="F72" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G72" s="1" t="inlineStr"/>
+      <c r="G72" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H72" s="1" t="inlineStr"/>
       <c r="I72" s="1" t="inlineStr"/>
       <c r="J72" s="1" t="inlineStr"/>
-      <c r="K72" s="1" t="inlineStr">
+      <c r="K72" s="1" t="inlineStr"/>
+      <c r="L72" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L72" s="1" t="inlineStr">
+      <c r="M72" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M72" s="1" t="inlineStr"/>
-      <c r="N72" s="1" t="inlineStr">
+      <c r="N72" s="1" t="inlineStr"/>
+      <c r="O72" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5416,22 +5634,25 @@
       <c r="F73" s="1" t="n">
         <v>995</v>
       </c>
-      <c r="G73" s="1" t="inlineStr"/>
+      <c r="G73" s="1" t="n">
+        <v>995</v>
+      </c>
       <c r="H73" s="1" t="inlineStr"/>
       <c r="I73" s="1" t="inlineStr"/>
       <c r="J73" s="1" t="inlineStr"/>
-      <c r="K73" s="1" t="inlineStr">
+      <c r="K73" s="1" t="inlineStr"/>
+      <c r="L73" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L73" s="1" t="inlineStr">
+      <c r="M73" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M73" s="1" t="inlineStr"/>
-      <c r="N73" s="1" t="inlineStr">
+      <c r="N73" s="1" t="inlineStr"/>
+      <c r="O73" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5466,22 +5687,25 @@
       <c r="F74" s="1" t="n">
         <v>149</v>
       </c>
-      <c r="G74" s="1" t="inlineStr"/>
+      <c r="G74" s="1" t="n">
+        <v>149</v>
+      </c>
       <c r="H74" s="1" t="inlineStr"/>
       <c r="I74" s="1" t="inlineStr"/>
       <c r="J74" s="1" t="inlineStr"/>
-      <c r="K74" s="1" t="inlineStr">
+      <c r="K74" s="1" t="inlineStr"/>
+      <c r="L74" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L74" s="1" t="inlineStr">
+      <c r="M74" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M74" s="1" t="inlineStr"/>
-      <c r="N74" s="1" t="inlineStr">
+      <c r="N74" s="1" t="inlineStr"/>
+      <c r="O74" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5516,22 +5740,25 @@
       <c r="F75" t="n">
         <v>349</v>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="n">
+        <v>349</v>
+      </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr">
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="M75" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr">
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5566,22 +5793,25 @@
       <c r="F76" t="n">
         <v>199</v>
       </c>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="n">
+        <v>199</v>
+      </c>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr">
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr">
+      <c r="M76" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr">
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5616,22 +5846,25 @@
       <c r="F77" t="n">
         <v>199</v>
       </c>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="n">
+        <v>199</v>
+      </c>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr">
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="M77" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr">
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5666,22 +5899,25 @@
       <c r="F78" t="n">
         <v>349</v>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="n">
+        <v>349</v>
+      </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr">
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="M78" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr">
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5716,22 +5952,25 @@
       <c r="F79" t="n">
         <v>399</v>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="n">
+        <v>399</v>
+      </c>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr">
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="M79" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr">
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5766,22 +6005,25 @@
       <c r="F80" t="n">
         <v>2249</v>
       </c>
-      <c r="G80" t="inlineStr"/>
+      <c r="G80" t="n">
+        <v>2249</v>
+      </c>
       <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr">
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr">
+      <c r="M80" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr">
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5816,22 +6058,25 @@
       <c r="F81" t="n">
         <v>249</v>
       </c>
-      <c r="G81" t="inlineStr"/>
+      <c r="G81" t="n">
+        <v>249</v>
+      </c>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr">
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr">
+      <c r="M81" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr">
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5866,22 +6111,25 @@
       <c r="F82" t="n">
         <v>199</v>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="G82" t="n">
+        <v>199</v>
+      </c>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr">
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr">
+      <c r="M82" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr">
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5916,22 +6164,25 @@
       <c r="F83" t="n">
         <v>299</v>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="G83" t="n">
+        <v>299</v>
+      </c>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr">
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr">
+      <c r="M83" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr">
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5966,22 +6217,25 @@
       <c r="F84" t="n">
         <v>225</v>
       </c>
-      <c r="G84" t="inlineStr"/>
+      <c r="G84" t="n">
+        <v>225</v>
+      </c>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr">
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr">
+      <c r="M84" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr">
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -6016,22 +6270,25 @@
       <c r="F85" t="n">
         <v>275</v>
       </c>
-      <c r="G85" t="inlineStr"/>
+      <c r="G85" t="n">
+        <v>275</v>
+      </c>
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr">
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="M85" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr">
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -6066,22 +6323,25 @@
       <c r="F86" t="n">
         <v>1199</v>
       </c>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="n">
+        <v>1199</v>
+      </c>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr">
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
+      <c r="M86" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr">
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -6116,22 +6376,25 @@
       <c r="F87" t="n">
         <v>349</v>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="n">
+        <v>349</v>
+      </c>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr">
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr">
+      <c r="M87" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr">
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Group foot care products under Insoles category in report
</commit_message>
<xml_diff>
--- a/full_product_variants_report.xlsx
+++ b/full_product_variants_report.xlsx
@@ -5712,532 +5712,532 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Brush &amp; Pumice Combo Turqouise</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-brush-pumice-combo-turqouise-def</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
+      <c r="D75" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E75" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-brush-pumice-combo-turqouise</t>
         </is>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="1" t="n">
         <v>349</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G75" s="1" t="n">
         <v>349</v>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr">
+      <c r="H75" s="1" t="inlineStr"/>
+      <c r="I75" s="1" t="inlineStr"/>
+      <c r="J75" s="1" t="inlineStr"/>
+      <c r="K75" s="1" t="inlineStr"/>
+      <c r="L75" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="M75" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N75" s="1" t="inlineStr"/>
+      <c r="O75" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Double sided Foot File Pink</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-double-sided-foot-file-pink-defa</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D76" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E76" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-double-sided-foot-file-pink</t>
         </is>
       </c>
-      <c r="F76" t="n">
+      <c r="F76" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="G76" t="n">
+      <c r="G76" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr">
+      <c r="H76" s="1" t="inlineStr"/>
+      <c r="I76" s="1" t="inlineStr"/>
+      <c r="J76" s="1" t="inlineStr"/>
+      <c r="K76" s="1" t="inlineStr"/>
+      <c r="L76" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="M76" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N76" s="1" t="inlineStr"/>
+      <c r="O76" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Double sided Foot File Purple</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-double-sided-foot-file-purple-de</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D77" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E77" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-double-sided-foot-file-purple</t>
         </is>
       </c>
-      <c r="F77" t="n">
+      <c r="F77" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="G77" t="n">
+      <c r="G77" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr">
+      <c r="H77" s="1" t="inlineStr"/>
+      <c r="I77" s="1" t="inlineStr"/>
+      <c r="J77" s="1" t="inlineStr"/>
+      <c r="K77" s="1" t="inlineStr"/>
+      <c r="L77" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="M77" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N77" s="1" t="inlineStr"/>
+      <c r="O77" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Dual Action Foot File Turqouise</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-dual-action-foot-file-turqouise-</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
+      <c r="D78" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-dual-action-foot-file-turqouise</t>
         </is>
       </c>
-      <c r="F78" t="n">
+      <c r="F78" s="1" t="n">
         <v>349</v>
       </c>
-      <c r="G78" t="n">
+      <c r="G78" s="1" t="n">
         <v>349</v>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr">
+      <c r="H78" s="1" t="inlineStr"/>
+      <c r="I78" s="1" t="inlineStr"/>
+      <c r="J78" s="1" t="inlineStr"/>
+      <c r="K78" s="1" t="inlineStr"/>
+      <c r="L78" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="M78" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N78" s="1" t="inlineStr"/>
+      <c r="O78" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="1" t="inlineStr">
         <is>
           <t>PRO Essentials Magic Pedi Roller Pack Black</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-magic-pedi-roller-pack-black-def</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
+      <c r="D79" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E79" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-magic-pedi-roller-pack-black</t>
         </is>
       </c>
-      <c r="F79" t="n">
+      <c r="F79" s="1" t="n">
         <v>399</v>
       </c>
-      <c r="G79" t="n">
+      <c r="G79" s="1" t="n">
         <v>399</v>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr">
+      <c r="H79" s="1" t="inlineStr"/>
+      <c r="I79" s="1" t="inlineStr"/>
+      <c r="J79" s="1" t="inlineStr"/>
+      <c r="K79" s="1" t="inlineStr"/>
+      <c r="L79" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="M79" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N79" s="1" t="inlineStr"/>
+      <c r="O79" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="1" t="inlineStr">
         <is>
           <t>PRO Essentials Magic Pedi Roller</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-magic-pedi-roller-default</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
+      <c r="D80" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E80" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-magic-pedi-roller</t>
         </is>
       </c>
-      <c r="F80" t="n">
+      <c r="F80" s="1" t="n">
         <v>2249</v>
       </c>
-      <c r="G80" t="n">
+      <c r="G80" s="1" t="n">
         <v>2249</v>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr">
+      <c r="H80" s="1" t="inlineStr"/>
+      <c r="I80" s="1" t="inlineStr"/>
+      <c r="J80" s="1" t="inlineStr"/>
+      <c r="K80" s="1" t="inlineStr"/>
+      <c r="L80" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr">
+      <c r="M80" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N80" s="1" t="inlineStr"/>
+      <c r="O80" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Nail File Turqouise</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-nail-file-turqouise-default</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
+      <c r="D81" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E81" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-nail-file-turqouise</t>
         </is>
       </c>
-      <c r="F81" t="n">
+      <c r="F81" s="1" t="n">
         <v>249</v>
       </c>
-      <c r="G81" t="n">
+      <c r="G81" s="1" t="n">
         <v>249</v>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr">
+      <c r="H81" s="1" t="inlineStr"/>
+      <c r="I81" s="1" t="inlineStr"/>
+      <c r="J81" s="1" t="inlineStr"/>
+      <c r="K81" s="1" t="inlineStr"/>
+      <c r="L81" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="M81" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N81" s="1" t="inlineStr"/>
+      <c r="O81" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Nail Buffer Turqouise</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-nail-buffer-turqouise-default</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D82" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E82" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-nail-buffer-turqouise</t>
         </is>
       </c>
-      <c r="F82" t="n">
+      <c r="F82" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="G82" t="n">
+      <c r="G82" s="1" t="n">
         <v>199</v>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr">
+      <c r="H82" s="1" t="inlineStr"/>
+      <c r="I82" s="1" t="inlineStr"/>
+      <c r="J82" s="1" t="inlineStr"/>
+      <c r="K82" s="1" t="inlineStr"/>
+      <c r="L82" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr">
+      <c r="M82" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N82" s="1" t="inlineStr"/>
+      <c r="O82" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Nail Clipper Turqouise</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-nail-clipper-turqouise-default</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
+      <c r="D83" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E83" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-nail-clipper-turqouise</t>
         </is>
       </c>
-      <c r="F83" t="n">
+      <c r="F83" s="1" t="n">
         <v>299</v>
       </c>
-      <c r="G83" t="n">
+      <c r="G83" s="1" t="n">
         <v>299</v>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr">
+      <c r="H83" s="1" t="inlineStr"/>
+      <c r="I83" s="1" t="inlineStr"/>
+      <c r="J83" s="1" t="inlineStr"/>
+      <c r="K83" s="1" t="inlineStr"/>
+      <c r="L83" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr">
+      <c r="M83" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N83" s="1" t="inlineStr"/>
+      <c r="O83" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="1" t="inlineStr">
         <is>
           <t>Pro Essentials Smooth Feet Pumice Turqouise</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="1" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="1" t="inlineStr">
         <is>
           <t>PG-pro-essentials-smooth-feet-pumice-turqouise-def</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
+      <c r="D84" s="1" t="inlineStr">
+        <is>
+          <t>Insoles</t>
+        </is>
+      </c>
+      <c r="E84" s="1" t="inlineStr">
         <is>
           <t>https://shop.mvshoecare.com/products/pro-essentials-smooth-feet-pumice-turqouise</t>
         </is>
       </c>
-      <c r="F84" t="n">
+      <c r="F84" s="1" t="n">
         <v>225</v>
       </c>
-      <c r="G84" t="n">
+      <c r="G84" s="1" t="n">
         <v>225</v>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr">
+      <c r="H84" s="1" t="inlineStr"/>
+      <c r="I84" s="1" t="inlineStr"/>
+      <c r="J84" s="1" t="inlineStr"/>
+      <c r="K84" s="1" t="inlineStr"/>
+      <c r="L84" s="1" t="inlineStr">
         <is>
           <t>Free Shipping, 30 Day Return, Eco Friendly, Complete Kit</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="M84" s="1" t="inlineStr">
         <is>
           <t>/images/polish.jpeg</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="N84" s="1" t="inlineStr"/>
+      <c r="O84" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>